<commit_message>
feat: extract vocab for rulebase
</commit_message>
<xml_diff>
--- a/data/raw/user_questions/QA_datasets.xlsx
+++ b/data/raw/user_questions/QA_datasets.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IT\THI\PAPER\project\neurosymbolic-legal-reasoner\data\raw\user_questions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCF4E899-359C-4905-9A43-289394AE7F8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FAE33D5-7F57-4686-B91E-7B2DDCAAE9CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1835,7 +1835,7 @@
   <cols>
     <col min="1" max="1" width="24.77734375" style="6" customWidth="1"/>
     <col min="2" max="2" width="21.44140625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="183.77734375" style="6" customWidth="1"/>
+    <col min="3" max="3" width="53.88671875" style="6" customWidth="1"/>
     <col min="4" max="4" width="20.33203125" style="6" customWidth="1"/>
     <col min="5" max="5" width="59" style="6" customWidth="1"/>
     <col min="6" max="16384" width="8.88671875" style="6"/>
@@ -1888,7 +1888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="228" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="216" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>14</v>
       </c>
@@ -1933,7 +1933,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="336" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5" ht="324" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
         <v>25</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="132" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" ht="120" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>40</v>
       </c>
@@ -2443,7 +2443,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="96" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:5" ht="84" x14ac:dyDescent="0.2">
       <c r="A41" s="3" t="s">
         <v>148</v>
       </c>
@@ -2488,7 +2488,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="108" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:5" ht="96" x14ac:dyDescent="0.2">
       <c r="A44" s="3" t="s">
         <v>160</v>
       </c>

</xml_diff>